<commit_message>
Retire the old catalogue and give each quotation a printable PDF
The 23 demo products and their images are gone; the 13 ProTech systems from
the ProtechInfo documents are the whole catalogue now.

Each of the four project quotations gains a one-page A4 PDF beside its
spreadsheet, generated by scripts/quotations-to-pdf.mjs. The .xlsx stays as
the editable source and the PDF is what the site offers first, so a price
change means editing one sheet and running `npm run quotations`.

The spreadsheets themselves needed repairing: their zip entries were named
with backslashes (xl\worksheets\sheet1.xml), which is not a valid OPC part
name, so the relationship pointing at worksheets/sheet1.xml resolved to
nothing and Excel would not have found the sheet. Rewritten with the
separators the format requires.

Also drops the hardcoded WD Purple image branch in ProductDetail, whose
product and image files no longer exist.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/_quotations/ใบเสนอราคา_City Data Platform.xlsx
+++ b/public/files/_quotations/ใบเสนอราคา_City Data Platform.xlsx
@@ -1,20 +1,20 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <AppVersion>3.1</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="City Data Platform" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
-  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
-  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-08-11T17:32:17Z</dcterms:created>
-  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-08-11T17:32:17Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="10">
@@ -244,7 +244,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -527,22 +527,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="City Data Platform" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>